<commit_message>
Update to latest tested changes
</commit_message>
<xml_diff>
--- a/Dapur/TEMPLATE.xlsx
+++ b/Dapur/TEMPLATE.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adminF\Downloads\Lembar-Penagihan-Harian-main\Dapur\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\ADM IRC AND ZN\AA Lembar-Penagihan-Harian-main\Dapur\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{262308F6-5F0C-45F2-96FD-A892BEBBBCA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80CB855E-9028-47DD-A496-EF390DC594BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11760" xr2:uid="{97F4A87A-E423-475C-8EC9-EBD6A5C823E6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$B$1:$P$7</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -36,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t>Nama</t>
   </si>
@@ -92,9 +95,6 @@
     <t>Nilai Tunai</t>
   </si>
   <si>
-    <t>Keterangan</t>
-  </si>
-  <si>
     <t>TOTAL TAGIHAN</t>
   </si>
   <si>
@@ -122,26 +122,28 @@
     <t>YY-SHINTA</t>
   </si>
   <si>
-    <t>YY-5758</t>
-  </si>
-  <si>
-    <t>17 Des 2025</t>
-  </si>
-  <si>
     <t>Rahvayana</t>
   </si>
   <si>
     <t>888 hari</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YY-5758 </t>
+  </si>
+  <si>
+    <t>Tgl</t>
+  </si>
+  <si>
+    <t>Ket</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="d/m/yyyy"/>
-    <numFmt numFmtId="165" formatCode="[$Rp-421]#,##0"/>
-    <numFmt numFmtId="166" formatCode="@\ * \:"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="[$Rp-421]#,##0"/>
+    <numFmt numFmtId="165" formatCode="@\ * \:"/>
   </numFmts>
   <fonts count="12">
     <font>
@@ -356,7 +358,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -365,7 +367,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -380,9 +382,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -409,9 +408,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="14" fontId="7" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -430,20 +426,35 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -462,8 +473,20 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -801,55 +824,63 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F287CAE-6193-48A8-89CC-ACC8E7E93C93}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:P7"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="9" style="2"/>
     <col min="2" max="2" width="11.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.7109375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="97.7109375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="25.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.7109375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="65.7109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="18.7109375" style="1" customWidth="1"/>
     <col min="6" max="6" width="34.7109375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="50.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="10" width="41.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="16" width="37.7109375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="32.140625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="41.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="39.7109375" style="1" customWidth="1"/>
+    <col min="11" max="11" width="28.7109375" style="1" customWidth="1"/>
+    <col min="12" max="12" width="37.7109375" style="1" customWidth="1"/>
+    <col min="13" max="13" width="28.7109375" style="1" customWidth="1"/>
+    <col min="14" max="15" width="37.7109375" style="1" customWidth="1"/>
+    <col min="16" max="16" width="30.7109375" style="1" customWidth="1"/>
     <col min="17" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="5" customFormat="1" ht="44.25">
+    <row r="1" spans="1:16" s="5" customFormat="1" ht="75" customHeight="1">
       <c r="A1" s="3"/>
-      <c r="B1" s="32" t="s">
-        <v>24</v>
-      </c>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
-      <c r="I1" s="32"/>
-      <c r="J1" s="32"/>
-      <c r="K1" s="32"/>
-      <c r="L1" s="32"/>
-      <c r="M1" s="32"/>
-      <c r="N1" s="32"/>
-      <c r="O1" s="32"/>
-      <c r="P1" s="32"/>
+      <c r="B1" s="35" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
+      <c r="I1" s="35"/>
+      <c r="J1" s="35"/>
+      <c r="K1" s="35"/>
+      <c r="L1" s="35"/>
+      <c r="M1" s="35"/>
+      <c r="N1" s="35"/>
+      <c r="O1" s="35"/>
+      <c r="P1" s="35"/>
     </row>
-    <row r="2" spans="1:16" s="5" customFormat="1" ht="44.25">
+    <row r="2" spans="1:16" s="5" customFormat="1" ht="45" customHeight="1">
       <c r="A2" s="3"/>
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="34"/>
+      <c r="C2" s="37"/>
       <c r="D2" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="6" t="s">
+      <c r="F2" s="48" t="s">
         <v>1</v>
       </c>
+      <c r="G2" s="48"/>
       <c r="H2" s="8" t="s">
         <v>2</v>
       </c>
@@ -858,178 +889,178 @@
         <v>3</v>
       </c>
       <c r="K2" s="10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M2" s="4"/>
       <c r="N2" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="O2" s="11">
+      <c r="O2" s="28">
         <v>46119</v>
       </c>
       <c r="P2" s="4"/>
     </row>
-    <row r="3" spans="1:16" s="5" customFormat="1" ht="44.25">
+    <row r="3" spans="1:16" s="5" customFormat="1" ht="45" customHeight="1">
       <c r="A3" s="3"/>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
       <c r="D3" s="4"/>
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
-      <c r="G3" s="12"/>
-      <c r="H3" s="13"/>
-      <c r="I3" s="13"/>
-      <c r="J3" s="13"/>
-      <c r="K3" s="14"/>
-      <c r="L3" s="14"/>
-      <c r="M3" s="41" t="s">
-        <v>23</v>
-      </c>
-      <c r="N3" s="41"/>
-      <c r="O3" s="15" t="s">
+      <c r="G3" s="11"/>
+      <c r="H3" s="12"/>
+      <c r="I3" s="12"/>
+      <c r="J3" s="12"/>
+      <c r="K3" s="13"/>
+      <c r="L3" s="13"/>
+      <c r="M3" s="44" t="s">
+        <v>22</v>
+      </c>
+      <c r="N3" s="44"/>
+      <c r="O3" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="P3" s="13"/>
+    </row>
+    <row r="4" spans="1:16" s="19" customFormat="1" ht="69.95" customHeight="1">
+      <c r="A4" s="15"/>
+      <c r="B4" s="16" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="G4" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="H4" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="I4" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="J4" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="K4" s="31" t="s">
+        <v>14</v>
+      </c>
+      <c r="L4" s="31" t="s">
+        <v>15</v>
+      </c>
+      <c r="M4" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="P3" s="14"/>
+      <c r="N4" s="31" t="s">
+        <v>16</v>
+      </c>
+      <c r="O4" s="31" t="s">
+        <v>17</v>
+      </c>
+      <c r="P4" s="18" t="s">
+        <v>31</v>
+      </c>
     </row>
-    <row r="4" spans="1:16" s="20" customFormat="1" ht="37.5">
-      <c r="A4" s="16"/>
-      <c r="B4" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" s="17" t="s">
-        <v>7</v>
-      </c>
-      <c r="E4" s="17" t="s">
-        <v>8</v>
-      </c>
-      <c r="F4" s="17" t="s">
-        <v>9</v>
-      </c>
-      <c r="G4" s="17" t="s">
-        <v>10</v>
-      </c>
-      <c r="H4" s="18" t="s">
-        <v>11</v>
-      </c>
-      <c r="I4" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="J4" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="K4" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="L4" s="19" t="s">
-        <v>15</v>
-      </c>
-      <c r="M4" s="19" t="s">
-        <v>4</v>
-      </c>
-      <c r="N4" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="O4" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="P4" s="19" t="s">
+    <row r="5" spans="1:16" s="19" customFormat="1" ht="75" customHeight="1">
+      <c r="A5" s="20"/>
+      <c r="B5" s="16">
+        <v>1</v>
+      </c>
+      <c r="C5" s="30" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" s="29" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" s="32" t="s">
+        <v>28</v>
+      </c>
+      <c r="F5" s="16">
+        <v>260500023</v>
+      </c>
+      <c r="G5" s="21">
+        <v>46186</v>
+      </c>
+      <c r="H5" s="22">
+        <v>1235758123</v>
+      </c>
+      <c r="I5" s="22">
+        <v>1231500000</v>
+      </c>
+      <c r="J5" s="23">
+        <v>1234258123</v>
+      </c>
+      <c r="K5" s="24"/>
+      <c r="L5" s="25"/>
+      <c r="M5" s="25"/>
+      <c r="N5" s="26"/>
+      <c r="O5" s="25"/>
+      <c r="P5" s="25"/>
+    </row>
+    <row r="6" spans="1:16" s="19" customFormat="1" ht="84.95" customHeight="1">
+      <c r="A6" s="15"/>
+      <c r="B6" s="45" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="5" spans="1:16" s="20" customFormat="1" ht="39">
-      <c r="A5" s="21"/>
-      <c r="B5" s="17">
-        <v>1</v>
-      </c>
-      <c r="C5" s="17" t="s">
-        <v>28</v>
-      </c>
-      <c r="D5" s="22" t="s">
-        <v>26</v>
-      </c>
-      <c r="E5" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="F5" s="17">
-        <v>260500023</v>
-      </c>
-      <c r="G5" s="23" t="s">
-        <v>29</v>
-      </c>
-      <c r="H5" s="24">
-        <v>1235758123</v>
-      </c>
-      <c r="I5" s="24">
-        <v>1231500000</v>
-      </c>
-      <c r="J5" s="25">
-        <v>1234258123</v>
-      </c>
-      <c r="K5" s="26"/>
-      <c r="L5" s="27"/>
-      <c r="M5" s="27"/>
-      <c r="N5" s="28"/>
-      <c r="O5" s="27"/>
-      <c r="P5" s="27"/>
-    </row>
-    <row r="6" spans="1:16" s="20" customFormat="1" ht="37.5">
-      <c r="A6" s="16"/>
-      <c r="B6" s="38" t="s">
-        <v>19</v>
-      </c>
-      <c r="C6" s="39"/>
-      <c r="D6" s="39"/>
-      <c r="E6" s="39"/>
-      <c r="F6" s="39"/>
-      <c r="G6" s="40"/>
-      <c r="H6" s="24">
+      <c r="C6" s="46"/>
+      <c r="D6" s="46"/>
+      <c r="E6" s="46"/>
+      <c r="F6" s="46"/>
+      <c r="G6" s="47"/>
+      <c r="H6" s="22">
         <f t="shared" ref="H6:I6" si="0">SUM(H5)</f>
         <v>1235758123</v>
       </c>
-      <c r="I6" s="24">
+      <c r="I6" s="22">
         <f t="shared" si="0"/>
         <v>1231500000</v>
       </c>
-      <c r="J6" s="25">
+      <c r="J6" s="23">
         <f>+SUM(J5)</f>
         <v>1234258123</v>
       </c>
-      <c r="K6" s="35" t="s">
+      <c r="K6" s="38" t="s">
+        <v>19</v>
+      </c>
+      <c r="L6" s="39"/>
+      <c r="M6" s="39"/>
+      <c r="N6" s="26"/>
+      <c r="O6" s="27"/>
+      <c r="P6" s="27"/>
+    </row>
+    <row r="7" spans="1:16" s="19" customFormat="1" ht="120" customHeight="1">
+      <c r="A7" s="15"/>
+      <c r="B7" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="L6" s="36"/>
-      <c r="M6" s="36"/>
-      <c r="N6" s="28"/>
-      <c r="O6" s="29"/>
-      <c r="P6" s="29"/>
-    </row>
-    <row r="7" spans="1:16" s="20" customFormat="1" ht="129.94999999999999" customHeight="1">
-      <c r="A7" s="16"/>
-      <c r="B7" s="38" t="s">
+      <c r="C7" s="42"/>
+      <c r="D7" s="42"/>
+      <c r="E7" s="42"/>
+      <c r="F7" s="42"/>
+      <c r="G7" s="42"/>
+      <c r="H7" s="42"/>
+      <c r="I7" s="42"/>
+      <c r="J7" s="43"/>
+      <c r="K7" s="40"/>
+      <c r="L7" s="34"/>
+      <c r="M7" s="40" t="s">
         <v>21</v>
       </c>
-      <c r="C7" s="39"/>
-      <c r="D7" s="39"/>
-      <c r="E7" s="39"/>
-      <c r="F7" s="39"/>
-      <c r="G7" s="39"/>
-      <c r="H7" s="39"/>
-      <c r="I7" s="39"/>
-      <c r="J7" s="40"/>
-      <c r="K7" s="37"/>
-      <c r="L7" s="31"/>
-      <c r="M7" s="37" t="s">
-        <v>22</v>
-      </c>
-      <c r="N7" s="31"/>
-      <c r="O7" s="30"/>
-      <c r="P7" s="31"/>
+      <c r="N7" s="34"/>
+      <c r="O7" s="33"/>
+      <c r="P7" s="34"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
     <mergeCell ref="O7:P7"/>
     <mergeCell ref="B1:P1"/>
     <mergeCell ref="B2:C2"/>
@@ -1039,7 +1070,9 @@
     <mergeCell ref="B7:J7"/>
     <mergeCell ref="M3:N3"/>
     <mergeCell ref="B6:G6"/>
+    <mergeCell ref="F2:G2"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="31" orientation="landscape" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>